<commit_message>
feat(corporate-pricing): land Override / New-Pricebook / Toolbar-IO + Search field-coverage
Lands the completed Corporate Pricing Wave-1.5 work (Product Group Override, New Pricebook create flow, Search toolbar Export/Import/Grid-Options, and Search field-coverage P2) plus the finished deliverable-workbook parity-recovery work (tc-parity guardrails, xlsx-lint rules, TestRail regen) — both share the regenerated workbook, so they land as one baseline. Internal plan-ID references stripped from the shipped test-data and spec comments.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients/encore/test_cases_xlsx/encore-qa-tracker.xlsx
+++ b/clients/encore/test_cases_xlsx/encore-qa-tracker.xlsx
@@ -3,9 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
-  <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500"/>
-  </bookViews>
   <sheets>
     <sheet sheetId="1" name="encore-qa-tracker" state="visible" r:id="rId4"/>
   </sheets>
@@ -14,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="171">
   <si>
     <t>COLOR KEY - our verification finding per item (rows sorted RED &gt; YELLOW &gt; GREEN within each Type section)</t>
   </si>
@@ -136,6 +133,33 @@
     <t>Delete should remain available so the row can be removed.</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
+    <t>Product bug</t>
+  </si>
+  <si>
+    <t>A10</t>
+  </si>
+  <si>
+    <t>Corporate Pricing - Pricing Detail (Max Discount column)</t>
+  </si>
+  <si>
+    <t>On the Pricing Detail tab of a price book, click into a Max Discount cell, type a value over 100 (e.g. 333), then try to click or tab out of the cell.</t>
+  </si>
+  <si>
+    <t>The field will not let you leave it — clicking elsewhere or pressing Tab does nothing and the cursor stays trapped in the cell. No error message, tooltip, or validation hint is shown. The only way out is to manually lower the value to 100 or less.</t>
+  </si>
+  <si>
+    <t>An out-of-range entry should show a clear validation message AND still let the user move out of the field — it should not silently trap the cursor with no feedback.</t>
+  </si>
+  <si>
+    <t>Out-of-range input appears to block the field’s blur/commit without surfacing a validation error.</t>
+  </si>
+  <si>
+    <t>Action required. Confirmed live by manual entry on the current site (2026-06-09). The 100% cap itself is reasonable; the defect is the silent focus-trap with no error and no way out.</t>
+  </si>
+  <si>
     <t>A1</t>
   </si>
   <si>
@@ -373,6 +397,51 @@
     <t>Should already-added locations be hidden from the dialog?</t>
   </si>
   <si>
+    <t>C4</t>
+  </si>
+  <si>
+    <t>Corporate Pricing - Pricing Detail (grid)</t>
+  </si>
+  <si>
+    <t>On the Pricing Detail tab of an existing price book, look for a way to expand a product-group row to see the items inside it.</t>
+  </si>
+  <si>
+    <t>The grid is flat — each product group is a single, non-expandable row with no way to drill into items. The written spec describes expanding a product group to show the items inside it.</t>
+  </si>
+  <si>
+    <t>Is the flat grid interim (the expandable group→items view still planned), or is the flat list the final design? Our coverage currently asserts the flat grid.</t>
+  </si>
+  <si>
+    <t>C5</t>
+  </si>
+  <si>
+    <t>Corporate Pricing - New Pricebook (Price Year)</t>
+  </si>
+  <si>
+    <t>On the New Pricebook form, type a decimal (e.g. 20.5) and a 2-digit value (e.g. 12) into Price Year, then try letters; check what is accepted and whether Save stays available.</t>
+  </si>
+  <si>
+    <t>Price Year rejects letters (the field reverts to the last valid value) but keeps a decimal (20.5) and a 2-digit value (12) without complaint. Server-side validation on final save was not exercised.</t>
+  </si>
+  <si>
+    <t>Should Price Year be restricted to a valid 4-digit year? Today only letters are blocked — 20.5 and 12 both pass the on-screen check.</t>
+  </si>
+  <si>
+    <t>C6</t>
+  </si>
+  <si>
+    <t>Corporate Pricing - New Pricebook (lifecycle)</t>
+  </si>
+  <si>
+    <t>Create and save a new price book, then look for any way to delete, deactivate, or remove it.</t>
+  </si>
+  <si>
+    <t>After a successful save there is no delete, deactivate, or remove option anywhere — not on the Details page, the Search action bar, any menu, or at row level. A created price book appears to be permanent via the UI.</t>
+  </si>
+  <si>
+    <t>Is there an intended way to remove or deactivate a price book created in error? This affects real-user error recovery.</t>
+  </si>
+  <si>
     <t>C1</t>
   </si>
   <si>
@@ -409,6 +478,24 @@
     <t>Testability / enablement request - submit separately from product bugs</t>
   </si>
   <si>
+    <t>D2</t>
+  </si>
+  <si>
+    <t>Corporate Pricing (all screens)</t>
+  </si>
+  <si>
+    <t>Inspect the Corporate Pricing screens for stable test identifiers.</t>
+  </si>
+  <si>
+    <t>The module ships with effectively no automation-grade test identifiers — Search has 3 generic ones; the Pricing Strategy, Pricing Detail, New Pricebook, Product Group Override, and Export/Import surfaces have none.</t>
+  </si>
+  <si>
+    <t>Stable, field-specific identifiers would make automated testing more reliable.</t>
+  </si>
+  <si>
+    <t>Testability / enablement request — a list of ~19 specific identifiers is provided separately. Please submit apart from the product items above.</t>
+  </si>
+  <si>
     <t>Test run summary</t>
   </si>
   <si>
@@ -425,6 +512,18 @@
   </si>
   <si>
     <t>Each item above was checked on both the current site and the previous Navigator version before being listed, so a genuine change can be told apart from long-standing behaviour.</t>
+  </si>
+  <si>
+    <t>This tracker lists 5 Corporate Pricing items raised by our testing: 1 confirmed defect (A10), 3 product/UX questions awaiting your answer (C4–C6), and 1 testability request (D2). Every item was re-checked live on the current site on 2026-06-09. A10 needs a fix; the 3 questions await a product decision; the testability request is enablement only.</t>
+  </si>
+  <si>
+    <t>Automated coverage for Corporate Pricing spans the Search page, the Pricebook Details page (both the Pricing Strategy and Pricing Detail tabs), the New Pricebook create flow, the Product Group Override screen, and the Search Export/Import toolbar. These checks run against the current site and pass.</t>
+  </si>
+  <si>
+    <t>Each item above was checked on the current site before being listed. Corporate Pricing is a new module with no equivalent on the previous Navigator version, so there is no older site to compare against; the written feature spec is used as the reference for intended behaviour, and anything we could not resolve from it is raised above as a question.</t>
+  </si>
+  <si>
+    <t>Not yet covered / paused: the full file-content round-trip for Export/Import — the on-screen triggers (the four Export/Import variants) are covered, but the exported/imported file contents depend on that feature stabilising.</t>
   </si>
 </sst>
 </file>
@@ -475,11 +574,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -508,44 +616,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -573,31 +681,14 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -625,23 +716,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -653,136 +727,180 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
+                <a:tint val="100000"/>
                 <a:shade val="100000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
-            <a:schemeClr val="phClr"/>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
     <a:lnDef>
       <a:spPr/>
       <a:bodyPr/>
@@ -804,18 +922,13 @@
     </a:lnDef>
   </a:objectDefaults>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I34"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
+  <dimension ref="A1:I43"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -980,30 +1093,32 @@
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="3"/>
-      <c r="B12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="A12" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D12" t="s">
-        <v>23</v>
-      </c>
-      <c r="E12" t="s">
+      <c r="B12" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="F12" t="s">
+      <c r="C12" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="G12" t="s">
+      <c r="D12" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="H12" t="s">
+      <c r="E12" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I12" t="s">
-        <v>34</v>
+      <c r="F12" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -1012,22 +1127,22 @@
         <v>14</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D13" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="E13" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F13" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G13" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="H13" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="I13" t="s">
         <v>34</v>
@@ -1039,22 +1154,22 @@
         <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D14" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E14" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F14" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H14" t="s">
-        <v>20</v>
+        <v>59</v>
       </c>
       <c r="I14" t="s">
         <v>34</v>
@@ -1066,19 +1181,19 @@
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D15" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="E15" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="F15" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="G15" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="H15" t="s">
         <v>20</v>
@@ -1093,381 +1208,577 @@
         <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D16" t="s">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="E16" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F16" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="G16" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="H16" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="I16" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
+      <c r="A17" s="3"/>
       <c r="B17" t="s">
-        <v>66</v>
+        <v>14</v>
       </c>
       <c r="C17" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D17" t="s">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="E17" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F17" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H17" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="I17" t="s">
-        <v>72</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="C18" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D18" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="E18" t="s">
+        <v>78</v>
+      </c>
+      <c r="F18" t="s">
+        <v>79</v>
+      </c>
+      <c r="G18" t="s">
+        <v>80</v>
+      </c>
+      <c r="H18" t="s">
+        <v>20</v>
+      </c>
+      <c r="I18" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="1"/>
+      <c r="B19" t="s">
         <v>75</v>
       </c>
-      <c r="F18" t="s">
-        <v>76</v>
-      </c>
-      <c r="G18" t="s">
-        <v>77</v>
-      </c>
-      <c r="H18" t="s">
-        <v>20</v>
-      </c>
-      <c r="I18" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
-      <c r="B19" t="s">
-        <v>66</v>
-      </c>
       <c r="C19" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D19" t="s">
-        <v>46</v>
+        <v>83</v>
       </c>
       <c r="E19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="F19" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="G19" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="H19" t="s">
         <v>20</v>
       </c>
       <c r="I19" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="C20" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D20" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="E20" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F20" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G20" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="H20" t="s">
         <v>20</v>
       </c>
       <c r="I20" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="C21" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D21" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="E21" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F21" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G21" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H21" t="s">
         <v>20</v>
       </c>
       <c r="I21" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="C22" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D22" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="E22" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="F22" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="G22" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="H22" t="s">
         <v>20</v>
       </c>
       <c r="I22" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="3"/>
+      <c r="A23" s="2"/>
       <c r="B23" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="C23" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D23" t="s">
-        <v>100</v>
+        <v>55</v>
       </c>
       <c r="E23" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="F23" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G23" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="H23" t="s">
         <v>20</v>
       </c>
       <c r="I23" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="C24" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D24" t="s">
+        <v>109</v>
+      </c>
+      <c r="E24" t="s">
+        <v>110</v>
+      </c>
+      <c r="F24" t="s">
+        <v>111</v>
+      </c>
+      <c r="G24" t="s">
+        <v>112</v>
+      </c>
+      <c r="H24" t="s">
+        <v>20</v>
+      </c>
+      <c r="I24" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="3"/>
+      <c r="B25" t="s">
+        <v>75</v>
+      </c>
+      <c r="C25" t="s">
+        <v>114</v>
+      </c>
+      <c r="D25" t="s">
         <v>36</v>
       </c>
-      <c r="E24" t="s">
-        <v>106</v>
-      </c>
-      <c r="F24" t="s">
-        <v>107</v>
-      </c>
-      <c r="G24" t="s">
-        <v>108</v>
-      </c>
-      <c r="H24" t="s">
-        <v>20</v>
-      </c>
-      <c r="I24" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="2"/>
-      <c r="B25" t="s">
-        <v>109</v>
-      </c>
-      <c r="C25" t="s">
-        <v>110</v>
-      </c>
-      <c r="D25" t="s">
-        <v>46</v>
-      </c>
       <c r="E25" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="F25" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="G25" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="H25" t="s">
         <v>20</v>
       </c>
       <c r="I25" t="s">
-        <v>114</v>
+        <v>92</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
       <c r="B26" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="C26" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D26" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="E26" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="F26" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="G26" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="H26" t="s">
         <v>20</v>
       </c>
       <c r="I26" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="2"/>
+      <c r="B27" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="3"/>
-      <c r="B27" t="s">
-        <v>109</v>
-      </c>
       <c r="C27" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D27" t="s">
-        <v>120</v>
+        <v>77</v>
       </c>
       <c r="E27" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="F27" t="s">
+        <v>126</v>
+      </c>
+      <c r="G27" t="s">
         <v>122</v>
       </c>
-      <c r="G27" t="s">
-        <v>113</v>
-      </c>
       <c r="H27" t="s">
         <v>20</v>
       </c>
       <c r="I27" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B28" t="s">
-        <v>124</v>
-      </c>
-      <c r="C28" t="s">
-        <v>125</v>
-      </c>
-      <c r="D28" t="s">
-        <v>126</v>
-      </c>
-      <c r="E28" t="s">
         <v>127</v>
       </c>
-      <c r="F28" t="s">
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="G28" t="s">
+      <c r="D28" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="H28" t="s">
-        <v>20</v>
-      </c>
-      <c r="I28" t="s">
+      <c r="E28" s="5" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+      <c r="F28" s="5" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+      <c r="G28" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I28" s="5" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C29" s="5" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="D29" s="5" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+      <c r="E29" s="5" t="s">
         <v>135</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="3"/>
+      <c r="B31" t="s">
+        <v>118</v>
+      </c>
+      <c r="C31" t="s">
+        <v>143</v>
+      </c>
+      <c r="D31" t="s">
+        <v>144</v>
+      </c>
+      <c r="E31" t="s">
+        <v>145</v>
+      </c>
+      <c r="F31" t="s">
+        <v>146</v>
+      </c>
+      <c r="G31" t="s">
+        <v>122</v>
+      </c>
+      <c r="H31" t="s">
+        <v>20</v>
+      </c>
+      <c r="I31" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>148</v>
+      </c>
+      <c r="C32" t="s">
+        <v>149</v>
+      </c>
+      <c r="D32" t="s">
+        <v>150</v>
+      </c>
+      <c r="E32" t="s">
+        <v>151</v>
+      </c>
+      <c r="F32" t="s">
+        <v>152</v>
+      </c>
+      <c r="G32" t="s">
+        <v>153</v>
+      </c>
+      <c r="H32" t="s">
+        <v>20</v>
+      </c>
+      <c r="I32" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="H33" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>136</v>
-      </c>
+        <v>161</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="B40" s="5"/>
+      <c r="C40" s="5"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5"/>
+      <c r="I40" s="5"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="B41" s="5"/>
+      <c r="C41" s="5"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5"/>
+      <c r="I41" s="5"/>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="B42" s="5"/>
+      <c r="C42" s="5"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
+      <c r="G42" s="5"/>
+      <c r="H42" s="5"/>
+      <c r="I42" s="5"/>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="B43" s="5"/>
+      <c r="C43" s="5"/>
+      <c r="D43" s="5"/>
+      <c r="E43" s="5"/>
+      <c r="F43" s="5"/>
+      <c r="G43" s="5"/>
+      <c r="H43" s="5"/>
+      <c r="I43" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(corp-pricing): NM-2263 New-Pricebook + coverage-followups + Labor Save/route-parity gate
- New-Pricebook (Labor+Equipment): TC-CPR-NPB-031..052 incl. Labor Save positive-control (051/052)
- Strategy: TC-CPR-STR-013 rewritten as a self-seeded cross-surface integration test (no vacuous pass)
- New gates: check-vacuous-grid-assertions (warn-only), check-save-route-parity (LR-066)
- Account & Address: 8 search-dialog TCs flipped Pass->Blocked in the deliverable per confirmed
  BUG-LOC-ACC-002 (backend account-search returns empty for every query); curated client-facing
  reasons added to blocked-reasons.json
- Rebuilt encore_test_cases.xlsx from source; removed redundant temp corp-pricing tracker (fully
  duplicated in encore-qa-tracker.xlsx)
- Plans NM2263 / Coverage-Followups / Labor-Save moved to done/
</commit_message>
<xml_diff>
--- a/clients/encore/test_cases_xlsx/encore-qa-tracker.xlsx
+++ b/clients/encore/test_cases_xlsx/encore-qa-tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="178">
   <si>
     <t>COLOR KEY - our verification finding per item (rows sorted RED &gt; YELLOW &gt; GREEN within each Type section)</t>
   </si>
@@ -160,6 +160,27 @@
     <t>Action required. Confirmed live by manual entry on the current site (2026-06-09). The 100% cap itself is reasonable; the defect is the silent focus-trap with no error and no way out.</t>
   </si>
   <si>
+    <t>A11</t>
+  </si>
+  <si>
+    <t>Corporate Pricing - Pricing Detail (New Price column)</t>
+  </si>
+  <si>
+    <t>On the Pricing Detail tab of a price book, click into a New Price cell, type an out-of-range value (e.g. 5646464), then commit it so the cell shows its error state.</t>
+  </si>
+  <si>
+    <t>As the red error icon appears, the number you typed shifts to the left to make room for the icon — the value visibly jumps sideways. The red border and icon otherwise render correctly and the value is still rejected as expected.</t>
+  </si>
+  <si>
+    <t>The error border and icon should appear without moving the entered value — the number should stay in place and the icon should sit in its own reserved space.</t>
+  </si>
+  <si>
+    <t>The error icon appears to be inserted inline within the cell and pushes the value aside, rather than occupying reserved or overlaid space.</t>
+  </si>
+  <si>
+    <t>Action required (cosmetic). Confirmed live by manual observation on the current site (2026-06-26). Validation and the disabled-Save behaviour both work and no data is lost; the issue is purely the value jumping left when the error appears. The same inline-edit control is used by other editable price cells (e.g. Max Discount, Product Group Override), so the same shift may occur there too.</t>
+  </si>
+  <si>
     <t>A1</t>
   </si>
   <si>
@@ -514,7 +535,7 @@
     <t>Each item above was checked on both the current site and the previous Navigator version before being listed, so a genuine change can be told apart from long-standing behaviour.</t>
   </si>
   <si>
-    <t>This tracker lists 5 Corporate Pricing items raised by our testing: 1 confirmed defect (A10), 3 product/UX questions awaiting your answer (C4–C6), and 1 testability request (D2). Every item was re-checked live on the current site on 2026-06-09. A10 needs a fix; the 3 questions await a product decision; the testability request is enablement only.</t>
+    <t>This tracker lists 6 Corporate Pricing items raised by our testing: 2 confirmed defects (A10–A11), 3 product/UX questions awaiting your answer (C4–C6), and 1 testability request (D2). A10 (Max Discount focus-trap) and the question/testability items were re-checked live on 2026-06-09; A11 (New Price error-icon shift) was confirmed live on 2026-06-26. A10 and A11 need fixes; the 3 questions await a product decision; the testability request is enablement only.</t>
   </si>
   <si>
     <t>Automated coverage for Corporate Pricing spans the Search page, the Pricebook Details page (both the Pricing Strategy and Pricing Detail tabs), the New Pricebook create flow, the Product Group Override screen, and the Search Export/Import toolbar. These checks run against the current site and pass.</t>
@@ -927,30 +948,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1122,30 +1143,32 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="3"/>
-      <c r="B13" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="A13" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D13" t="s">
-        <v>23</v>
-      </c>
-      <c r="E13" t="s">
+      <c r="D13" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="F13" t="s">
+      <c r="E13" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="G13" t="s">
+      <c r="F13" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="H13" t="s">
+      <c r="G13" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="I13" t="s">
-        <v>34</v>
+      <c r="H13" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -1154,22 +1177,22 @@
         <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D14" t="s">
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="E14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G14" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H14" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I14" t="s">
         <v>34</v>
@@ -1181,22 +1204,22 @@
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E15" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F15" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H15" t="s">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="I15" t="s">
         <v>34</v>
@@ -1208,19 +1231,19 @@
         <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F16" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G16" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H16" t="s">
         <v>20</v>
@@ -1235,37 +1258,37 @@
         <v>14</v>
       </c>
       <c r="C17" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D17" t="s">
-        <v>36</v>
+        <v>73</v>
       </c>
       <c r="E17" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="F17" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="G17" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="H17" t="s">
-        <v>74</v>
+        <v>20</v>
       </c>
       <c r="I17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
+      <c r="A18" s="3"/>
       <c r="B18" t="s">
-        <v>75</v>
+        <v>14</v>
       </c>
       <c r="C18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D18" t="s">
-        <v>77</v>
+        <v>36</v>
       </c>
       <c r="E18" t="s">
         <v>78</v>
@@ -1277,282 +1300,280 @@
         <v>80</v>
       </c>
       <c r="H18" t="s">
-        <v>20</v>
+        <v>81</v>
       </c>
       <c r="I18" t="s">
-        <v>81</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C19" t="s">
+        <v>83</v>
+      </c>
+      <c r="D19" t="s">
+        <v>84</v>
+      </c>
+      <c r="E19" t="s">
+        <v>85</v>
+      </c>
+      <c r="F19" t="s">
+        <v>86</v>
+      </c>
+      <c r="G19" t="s">
+        <v>87</v>
+      </c>
+      <c r="H19" t="s">
+        <v>20</v>
+      </c>
+      <c r="I19" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="1"/>
+      <c r="B20" t="s">
         <v>82</v>
       </c>
-      <c r="D19" t="s">
-        <v>83</v>
-      </c>
-      <c r="E19" t="s">
-        <v>84</v>
-      </c>
-      <c r="F19" t="s">
-        <v>85</v>
-      </c>
-      <c r="G19" t="s">
-        <v>86</v>
-      </c>
-      <c r="H19" t="s">
-        <v>20</v>
-      </c>
-      <c r="I19" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
-      <c r="B20" t="s">
-        <v>75</v>
-      </c>
       <c r="C20" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D20" t="s">
-        <v>55</v>
+        <v>90</v>
       </c>
       <c r="E20" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F20" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G20" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H20" t="s">
         <v>20</v>
       </c>
       <c r="I20" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C21" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D21" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="E21" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F21" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G21" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H21" t="s">
         <v>20</v>
       </c>
       <c r="I21" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C22" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D22" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="E22" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F22" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G22" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H22" t="s">
         <v>20</v>
       </c>
       <c r="I22" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
       <c r="B23" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C23" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D23" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="E23" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F23" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G23" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="H23" t="s">
         <v>20</v>
       </c>
       <c r="I23" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="3"/>
+      <c r="A24" s="2"/>
       <c r="B24" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C24" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D24" t="s">
-        <v>109</v>
+        <v>62</v>
       </c>
       <c r="E24" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F24" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G24" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H24" t="s">
         <v>20</v>
       </c>
       <c r="I24" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C25" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D25" t="s">
+        <v>116</v>
+      </c>
+      <c r="E25" t="s">
+        <v>117</v>
+      </c>
+      <c r="F25" t="s">
+        <v>118</v>
+      </c>
+      <c r="G25" t="s">
+        <v>119</v>
+      </c>
+      <c r="H25" t="s">
+        <v>20</v>
+      </c>
+      <c r="I25" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="3"/>
+      <c r="B26" t="s">
+        <v>82</v>
+      </c>
+      <c r="C26" t="s">
+        <v>121</v>
+      </c>
+      <c r="D26" t="s">
         <v>36</v>
       </c>
-      <c r="E25" t="s">
-        <v>115</v>
-      </c>
-      <c r="F25" t="s">
-        <v>116</v>
-      </c>
-      <c r="G25" t="s">
-        <v>117</v>
-      </c>
-      <c r="H25" t="s">
-        <v>20</v>
-      </c>
-      <c r="I25" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="2"/>
-      <c r="B26" t="s">
-        <v>118</v>
-      </c>
-      <c r="C26" t="s">
-        <v>119</v>
-      </c>
-      <c r="D26" t="s">
-        <v>55</v>
-      </c>
       <c r="E26" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F26" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G26" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H26" t="s">
         <v>20</v>
       </c>
       <c r="I26" t="s">
-        <v>123</v>
+        <v>99</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="C27" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D27" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="E27" t="s">
+        <v>127</v>
+      </c>
+      <c r="F27" t="s">
+        <v>128</v>
+      </c>
+      <c r="G27" t="s">
+        <v>129</v>
+      </c>
+      <c r="H27" t="s">
+        <v>20</v>
+      </c>
+      <c r="I27" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="2"/>
+      <c r="B28" t="s">
         <v>125</v>
       </c>
-      <c r="F27" t="s">
-        <v>126</v>
-      </c>
-      <c r="G27" t="s">
-        <v>122</v>
-      </c>
-      <c r="H27" t="s">
-        <v>20</v>
-      </c>
-      <c r="I27" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="D28" s="5" t="s">
+      <c r="C28" t="s">
+        <v>131</v>
+      </c>
+      <c r="D28" t="s">
+        <v>84</v>
+      </c>
+      <c r="E28" t="s">
+        <v>132</v>
+      </c>
+      <c r="F28" t="s">
+        <v>133</v>
+      </c>
+      <c r="G28" t="s">
         <v>129</v>
       </c>
-      <c r="E28" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="H28" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="I28" s="5" t="s">
-        <v>132</v>
+      <c r="H28" t="s">
+        <v>20</v>
+      </c>
+      <c r="I28" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -1560,28 +1581,28 @@
         <v>40</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="H29" s="5" t="s">
         <v>20</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -1589,75 +1610,78 @@
         <v>40</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="H30" s="5" t="s">
         <v>20</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="3"/>
-      <c r="B31" t="s">
-        <v>118</v>
-      </c>
-      <c r="C31" t="s">
-        <v>143</v>
-      </c>
-      <c r="D31" t="s">
-        <v>144</v>
-      </c>
-      <c r="E31" t="s">
+      <c r="A31" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C31" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="F31" t="s">
+      <c r="D31" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="G31" t="s">
-        <v>122</v>
-      </c>
-      <c r="H31" t="s">
-        <v>20</v>
-      </c>
-      <c r="I31" t="s">
+      <c r="E31" s="5" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="F31" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I31" s="5" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="3"/>
       <c r="B32" t="s">
-        <v>148</v>
+        <v>125</v>
       </c>
       <c r="C32" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D32" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E32" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F32" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G32" t="s">
-        <v>153</v>
+        <v>129</v>
       </c>
       <c r="H32" t="s">
         <v>20</v>
@@ -1667,80 +1691,93 @@
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="5" t="s">
+      <c r="B33" t="s">
+        <v>155</v>
+      </c>
+      <c r="C33" t="s">
+        <v>156</v>
+      </c>
+      <c r="D33" t="s">
+        <v>157</v>
+      </c>
+      <c r="E33" t="s">
+        <v>158</v>
+      </c>
+      <c r="F33" t="s">
+        <v>159</v>
+      </c>
+      <c r="G33" t="s">
+        <v>160</v>
+      </c>
+      <c r="H33" t="s">
+        <v>20</v>
+      </c>
+      <c r="I33" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B33" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="C33" s="5" t="s">
+      <c r="B34" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="D33" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="E33" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="F33" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="H33" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="I33" s="5" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="C34" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="B40" s="5"/>
-      <c r="C40" s="5"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
-      <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
-      <c r="I40" s="5"/>
+        <v>172</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>173</v>
+      </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="B41" s="5"/>
       <c r="C41" s="5"/>
@@ -1753,7 +1790,7 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="B42" s="5"/>
       <c r="C42" s="5"/>
@@ -1766,7 +1803,7 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="B43" s="5"/>
       <c r="C43" s="5"/>
@@ -1777,6 +1814,19 @@
       <c r="H43" s="5"/>
       <c r="I43" s="5"/>
     </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="B44" s="5"/>
+      <c r="C44" s="5"/>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
+      <c r="H44" s="5"/>
+      <c r="I44" s="5"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
feat(corp-pricing): re-anchor Override fixture to office 1606 + file 1604 data/import defect
Office 1604's Product Group Override grid reads empty while a same-screen Export
lists 8 rows, and imports fail server-side (duplicate-key "4543" or silent
no-persist). Re-anchored the fixture 1604 -> 1606 (healthy control; 28 passed /
1 skipped) with a plain-English revert-to-1604 note embedding the original values.
Filed internal BUG-CPR-OVR-002 (baseline-absent) and added two client-facing rows
to encore-qa-tracker.xlsx: A12 (RED confirmed defect) + C7 (YELLOW data-restore
question); footer counts updated. Materialized PLAN_GATE_BACKLOG_AND_1604_TRACKER
(parent PLAN_ENCORE_DELIVERABLE_REMEDIATION Phase 5).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients/encore/test_cases_xlsx/encore-qa-tracker.xlsx
+++ b/clients/encore/test_cases_xlsx/encore-qa-tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="190">
   <si>
     <t>COLOR KEY - our verification finding per item (rows sorted RED &gt; YELLOW &gt; GREEN within each Type section)</t>
   </si>
@@ -181,6 +181,27 @@
     <t>Action required (cosmetic). Confirmed live by manual observation on the current site (2026-06-26). Validation and the disabled-Save behaviour both work and no data is lost; the issue is purely the value jumping left when the error appears. The same inline-edit control is used by other editable price cells (e.g. Max Discount, Product Group Override), so the same shift may occur there too.</t>
   </si>
   <si>
+    <t>A12</t>
+  </si>
+  <si>
+    <t>Corporate Pricing - Product Group Override (office 1604 data &amp; import)</t>
+  </si>
+  <si>
+    <t>On the Product Group Override screen, select office 1604 in the Change Local Office picker. Then (a) click Export, and (b) try to import a price-override file for 1604 — first a file that includes the House Video Monitor product groups plus the Project Manager group, then a smaller file with only three House Video Monitor groups.</t>
+  </si>
+  <si>
+    <t>The grid shows "0 items found" for 1604, yet the Export of the same screen returns a file listing 8 override rows for 1604 — the grid and the export disagree. Importing a file that contains the Project Manager product group is rejected with a raw technical error ("An item with the same key has already been added. Key: 4543") instead of a readable message. Importing the smaller file reports "Override import complete. There were 3 override change updates.", but after reloading the grid is still empty — nothing was saved.</t>
+  </si>
+  <si>
+    <t>The grid and the Export of the same screen should agree for a location. An import should either save its rows (visible after reload) or reject them with a clear, readable message — never a raw internal error, and never a "success" message when nothing was saved.</t>
+  </si>
+  <si>
+    <t>Office 1604’s override data appears to be in an inconsistent server-side state that both hides existing rows from the grid and blocks new imports (the duplicate-key error even references a different location’s data).</t>
+  </si>
+  <si>
+    <t>Action required. Confirmed live on the current site (2026-07-06). Office 1606 works correctly on the same screen (7 rows shown, edit and save verified), so this looks specific to office 1604’s data. Our automated checks for this screen are pointed at office 1606 until this is resolved.</t>
+  </si>
+  <si>
     <t>A1</t>
   </si>
   <si>
@@ -463,6 +484,21 @@
     <t>Is there an intended way to remove or deactivate a price book created in error? This affects real-user error recovery.</t>
   </si>
   <si>
+    <t>C7</t>
+  </si>
+  <si>
+    <t>Corporate Pricing - Product Group Override (office 1604 data)</t>
+  </si>
+  <si>
+    <t>Compare office 1604’s override data over time: earlier testing (early June) saw override rows for 1604, and a same-day Export still lists 8 rows for it, but the grid now shows none.</t>
+  </si>
+  <si>
+    <t>Office 1604’s override grid is now empty, although the Export of the same screen still returns rows for it.</t>
+  </si>
+  <si>
+    <t>Was office 1604’s override data intentionally cleaned up or reset? If so, can it be restored or repopulated so that both the grid and the import work for that location again? This determines whether our checks can return to office 1604.</t>
+  </si>
+  <si>
     <t>C1</t>
   </si>
   <si>
@@ -535,7 +571,7 @@
     <t>Each item above was checked on both the current site and the previous Navigator version before being listed, so a genuine change can be told apart from long-standing behaviour.</t>
   </si>
   <si>
-    <t>This tracker lists 6 Corporate Pricing items raised by our testing: 2 confirmed defects (A10–A11), 3 product/UX questions awaiting your answer (C4–C6), and 1 testability request (D2). A10 (Max Discount focus-trap) and the question/testability items were re-checked live on 2026-06-09; A11 (New Price error-icon shift) was confirmed live on 2026-06-26. A10 and A11 need fixes; the 3 questions await a product decision; the testability request is enablement only.</t>
+    <t>This tracker lists 8 Corporate Pricing items raised by our testing: 3 confirmed defects (A10–A12), 4 product/UX questions awaiting your answer (C4–C7), and 1 testability request (D2). A10 (Max Discount focus-trap) and the question/testability items were re-checked live on 2026-06-09; A11 (New Price error-icon shift) was confirmed live on 2026-06-26; A12 (office 1604 override data/import) and C7 (office 1604 data-restore question) were confirmed live on 2026-07-06. A10, A11 and A12 need fixes; the 4 questions await a product decision; the testability request is enablement only.</t>
   </si>
   <si>
     <t>Automated coverage for Corporate Pricing spans the Search page, the Pricebook Details page (both the Pricing Strategy and Pricing Detail tabs), the New Pricebook create flow, the Product Group Override screen, and the Search Export/Import toolbar. These checks run against the current site and pass.</t>
@@ -948,7 +984,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -1172,30 +1208,30 @@
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="3"/>
-      <c r="B14" t="s">
-        <v>14</v>
-      </c>
-      <c r="C14" t="s">
+      <c r="A14" s="4"/>
+      <c r="B14" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D14" t="s">
-        <v>23</v>
-      </c>
-      <c r="E14" t="s">
+      <c r="D14" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="F14" t="s">
+      <c r="E14" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="G14" t="s">
+      <c r="F14" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="H14" t="s">
+      <c r="G14" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="I14" t="s">
-        <v>34</v>
+      <c r="H14" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -1204,22 +1240,22 @@
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D15" t="s">
-        <v>62</v>
+        <v>23</v>
       </c>
       <c r="E15" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G15" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H15" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I15" t="s">
         <v>34</v>
@@ -1231,22 +1267,22 @@
         <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D16" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E16" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F16" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G16" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H16" t="s">
-        <v>20</v>
+        <v>73</v>
       </c>
       <c r="I16" t="s">
         <v>34</v>
@@ -1258,19 +1294,19 @@
         <v>14</v>
       </c>
       <c r="C17" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D17" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E17" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F17" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G17" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H17" t="s">
         <v>20</v>
@@ -1285,37 +1321,37 @@
         <v>14</v>
       </c>
       <c r="C18" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D18" t="s">
-        <v>36</v>
+        <v>80</v>
       </c>
       <c r="E18" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F18" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G18" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="H18" t="s">
-        <v>81</v>
+        <v>20</v>
       </c>
       <c r="I18" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
+      <c r="A19" s="3"/>
       <c r="B19" t="s">
-        <v>82</v>
+        <v>14</v>
       </c>
       <c r="C19" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D19" t="s">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="E19" t="s">
         <v>85</v>
@@ -1327,282 +1363,280 @@
         <v>87</v>
       </c>
       <c r="H19" t="s">
-        <v>20</v>
+        <v>88</v>
       </c>
       <c r="I19" t="s">
-        <v>88</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C20" t="s">
+        <v>90</v>
+      </c>
+      <c r="D20" t="s">
+        <v>91</v>
+      </c>
+      <c r="E20" t="s">
+        <v>92</v>
+      </c>
+      <c r="F20" t="s">
+        <v>93</v>
+      </c>
+      <c r="G20" t="s">
+        <v>94</v>
+      </c>
+      <c r="H20" t="s">
+        <v>20</v>
+      </c>
+      <c r="I20" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="1"/>
+      <c r="B21" t="s">
         <v>89</v>
       </c>
-      <c r="D20" t="s">
-        <v>90</v>
-      </c>
-      <c r="E20" t="s">
-        <v>91</v>
-      </c>
-      <c r="F20" t="s">
-        <v>92</v>
-      </c>
-      <c r="G20" t="s">
-        <v>93</v>
-      </c>
-      <c r="H20" t="s">
-        <v>20</v>
-      </c>
-      <c r="I20" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="2"/>
-      <c r="B21" t="s">
-        <v>82</v>
-      </c>
       <c r="C21" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D21" t="s">
-        <v>62</v>
+        <v>97</v>
       </c>
       <c r="E21" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F21" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="G21" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H21" t="s">
         <v>20</v>
       </c>
       <c r="I21" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C22" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D22" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="E22" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F22" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G22" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H22" t="s">
         <v>20</v>
       </c>
       <c r="I22" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
       <c r="B23" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C23" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D23" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="E23" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F23" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G23" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="H23" t="s">
         <v>20</v>
       </c>
       <c r="I23" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C24" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D24" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="E24" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F24" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G24" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H24" t="s">
         <v>20</v>
       </c>
       <c r="I24" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="3"/>
+      <c r="A25" s="2"/>
       <c r="B25" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C25" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D25" t="s">
-        <v>116</v>
+        <v>69</v>
       </c>
       <c r="E25" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F25" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G25" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H25" t="s">
         <v>20</v>
       </c>
       <c r="I25" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C26" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D26" t="s">
+        <v>123</v>
+      </c>
+      <c r="E26" t="s">
+        <v>124</v>
+      </c>
+      <c r="F26" t="s">
+        <v>125</v>
+      </c>
+      <c r="G26" t="s">
+        <v>126</v>
+      </c>
+      <c r="H26" t="s">
+        <v>20</v>
+      </c>
+      <c r="I26" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="3"/>
+      <c r="B27" t="s">
+        <v>89</v>
+      </c>
+      <c r="C27" t="s">
+        <v>128</v>
+      </c>
+      <c r="D27" t="s">
         <v>36</v>
       </c>
-      <c r="E26" t="s">
-        <v>122</v>
-      </c>
-      <c r="F26" t="s">
-        <v>123</v>
-      </c>
-      <c r="G26" t="s">
-        <v>124</v>
-      </c>
-      <c r="H26" t="s">
-        <v>20</v>
-      </c>
-      <c r="I26" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="2"/>
-      <c r="B27" t="s">
-        <v>125</v>
-      </c>
-      <c r="C27" t="s">
-        <v>126</v>
-      </c>
-      <c r="D27" t="s">
-        <v>62</v>
-      </c>
       <c r="E27" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F27" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G27" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="H27" t="s">
         <v>20</v>
       </c>
       <c r="I27" t="s">
-        <v>130</v>
+        <v>106</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
       <c r="B28" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="C28" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D28" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="E28" t="s">
+        <v>134</v>
+      </c>
+      <c r="F28" t="s">
+        <v>135</v>
+      </c>
+      <c r="G28" t="s">
+        <v>136</v>
+      </c>
+      <c r="H28" t="s">
+        <v>20</v>
+      </c>
+      <c r="I28" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="2"/>
+      <c r="B29" t="s">
         <v>132</v>
       </c>
-      <c r="F28" t="s">
-        <v>133</v>
-      </c>
-      <c r="G28" t="s">
-        <v>129</v>
-      </c>
-      <c r="H28" t="s">
-        <v>20</v>
-      </c>
-      <c r="I28" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="D29" s="5" t="s">
+      <c r="C29" t="s">
+        <v>138</v>
+      </c>
+      <c r="D29" t="s">
+        <v>91</v>
+      </c>
+      <c r="E29" t="s">
+        <v>139</v>
+      </c>
+      <c r="F29" t="s">
+        <v>140</v>
+      </c>
+      <c r="G29" t="s">
         <v>136</v>
       </c>
-      <c r="E29" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="H29" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="I29" s="5" t="s">
-        <v>139</v>
+      <c r="H29" t="s">
+        <v>20</v>
+      </c>
+      <c r="I29" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -1610,28 +1644,28 @@
         <v>40</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="H30" s="5" t="s">
         <v>20</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -1639,171 +1673,201 @@
         <v>40</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="H31" s="5" t="s">
         <v>20</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="3"/>
-      <c r="B32" t="s">
-        <v>125</v>
-      </c>
-      <c r="C32" t="s">
-        <v>150</v>
-      </c>
-      <c r="D32" t="s">
-        <v>151</v>
-      </c>
-      <c r="E32" t="s">
+      <c r="A32" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C32" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="F32" t="s">
+      <c r="D32" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="G32" t="s">
-        <v>129</v>
-      </c>
-      <c r="H32" t="s">
-        <v>20</v>
-      </c>
-      <c r="I32" t="s">
+      <c r="E32" s="5" t="s">
         <v>154</v>
       </c>
+      <c r="F32" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I32" s="5" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B33" t="s">
-        <v>155</v>
-      </c>
-      <c r="C33" t="s">
-        <v>156</v>
-      </c>
-      <c r="D33" t="s">
+      <c r="A33" s="6"/>
+      <c r="B33" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C33" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="E33" t="s">
+      <c r="D33" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="F33" t="s">
+      <c r="E33" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="G33" t="s">
+      <c r="F33" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="H33" t="s">
-        <v>20</v>
-      </c>
-      <c r="I33" t="s">
+      <c r="G33" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="H33" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I33" s="5" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="5" t="s">
+      <c r="A34" s="3"/>
+      <c r="B34" t="s">
+        <v>132</v>
+      </c>
+      <c r="C34" t="s">
+        <v>162</v>
+      </c>
+      <c r="D34" t="s">
+        <v>163</v>
+      </c>
+      <c r="E34" t="s">
+        <v>164</v>
+      </c>
+      <c r="F34" t="s">
+        <v>165</v>
+      </c>
+      <c r="G34" t="s">
+        <v>136</v>
+      </c>
+      <c r="H34" t="s">
+        <v>20</v>
+      </c>
+      <c r="I34" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B35" t="s">
+        <v>167</v>
+      </c>
+      <c r="C35" t="s">
+        <v>168</v>
+      </c>
+      <c r="D35" t="s">
+        <v>169</v>
+      </c>
+      <c r="E35" t="s">
+        <v>170</v>
+      </c>
+      <c r="F35" t="s">
+        <v>171</v>
+      </c>
+      <c r="G35" t="s">
+        <v>172</v>
+      </c>
+      <c r="H35" t="s">
+        <v>20</v>
+      </c>
+      <c r="I35" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B34" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="E34" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="F34" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="G34" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="H34" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="I34" s="5" t="s">
+      <c r="B36" s="5" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>169</v>
+      <c r="C36" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I36" s="5" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="B41" s="5"/>
-      <c r="C41" s="5"/>
-      <c r="D41" s="5"/>
-      <c r="E41" s="5"/>
-      <c r="F41" s="5"/>
-      <c r="G41" s="5"/>
-      <c r="H41" s="5"/>
-      <c r="I41" s="5"/>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="B42" s="5"/>
-      <c r="C42" s="5"/>
-      <c r="D42" s="5"/>
-      <c r="E42" s="5"/>
-      <c r="F42" s="5"/>
-      <c r="G42" s="5"/>
-      <c r="H42" s="5"/>
-      <c r="I42" s="5"/>
+        <v>183</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>185</v>
+      </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="B43" s="5"/>
       <c r="C43" s="5"/>
@@ -1816,7 +1880,7 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="B44" s="5"/>
       <c r="C44" s="5"/>
@@ -1827,6 +1891,32 @@
       <c r="H44" s="5"/>
       <c r="I44" s="5"/>
     </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B45" s="5"/>
+      <c r="C45" s="5"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="5"/>
+      <c r="H45" s="5"/>
+      <c r="I45" s="5"/>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="B46" s="5"/>
+      <c r="C46" s="5"/>
+      <c r="D46" s="5"/>
+      <c r="E46" s="5"/>
+      <c r="F46" s="5"/>
+      <c r="G46" s="5"/>
+      <c r="H46" s="5"/>
+      <c r="I46" s="5"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>